<commit_message>
Improve OrangeHRM manual testing portfolio documentation
</commit_message>
<xml_diff>
--- a/05-Defect-Management/Bug-Reports.xlsx
+++ b/05-Defect-Management/Bug-Reports.xlsx
@@ -106,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -124,13 +124,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -500,24 +494,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="25" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="25" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -542,70 +538,80 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>Defect Title</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Module</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Reproducibility</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>Evidence Reference</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Comments</t>
         </is>
@@ -617,76 +623,86 @@
           <t>BUG_EMP_001</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Confirmed Defect</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Employee search by Employee Name fails when trailing whitespace is present in search input</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Employee Management (PIM)</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Demo</t>
-        </is>
-      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Employee 'Pranali Test' exists in the PIM Employee List.</t>
+          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Public Demo</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
+          <t>Active employee 'Pranali Test' exists in PIM Employee List.</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Employee Name: "Pranali " (with trailing whitespace)</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
           <t>1. Navigate to PIM &gt; Employee List.
-2. In the Employee Name input box, type 'Pranali ' (with a trailing space character).
-3. Click the 'Search' button.</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>System should trim leading and trailing whitespace automatically and return the matching record for 'Pranali Test'.</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>System displays 'No Records Found' toast notification because trailing whitespace is not sanitized prior to search lookup.</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
+2. In Employee Name search input box, type 'Pranali ' (with a trailing space).
+3. Click 'Search' button.</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>System should trim leading and trailing whitespace automatically and retrieve the matching record for 'Pranali Test'.</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>System queries literal string with space, fails to resolve autocomplete entry, and displays 'No Records Found'.</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Always (100%)</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>TC_EMP_009</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>BUG_EMP_001_trailing_space_search.png</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>Observed during manual exploratory testing. Affects user experience when copying and pasting names.</t>
+      <c r="Q5" s="5" t="inlineStr">
+        <is>
+          <t>Observed during manual exploratory testing. Affects real users who copy-paste names with accidental whitespace.</t>
         </is>
       </c>
     </row>
@@ -696,77 +712,87 @@
           <t>BUG_LEAVE_001</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Leave Date picker allows manual typing of past dates without immediate validation warning</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Confirmed Defect</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Leave Date picker allows manual entry of past dates without immediate validation warning</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Leave Management</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Demo</t>
-        </is>
-      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>User is on the Leave &gt; Apply page.</t>
+          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Public Demo</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>1. Select a valid Leave Type.
-2. Manually type a past date '2023-01-01' into From Date field.
-3. Type '2023-01-02' into To Date field.
+          <t>User is logged in and on Leave &gt; Apply page with allocated balance.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Leave Type: "US - Vacation", From Date: "2023-01-01", To Date: "2023-01-02"</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>1. Select active Leave Type.
+2. Manually enter past date '2023-01-01' into From Date field.
+3. Manually enter past date '2023-01-02' into To Date field.
 4. Click 'Apply' button.</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>System should immediately validate date fields and alert the user that leave cannot be requested for historical dates.</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>System does not validate past dates on client-side; form attempts submission and fails with a generic error banner.</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>System should validate date chronology against current system date and trigger inline warning: 'Leave cannot be applied for past dates'.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>UI accepts past dates without client-side warning; submission attempts processing and returns generic server error banner.</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="J6" s="7" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Always (100%)</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="N6" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>TC_LEAVE_002</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>BUG_LEAVE_001_past_date_warning.png</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Past date validation logic should be handled with explicit error messaging on the UI.</t>
+      <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>Client-side boundary validation missing on manual text entry for date picker fields.</t>
         </is>
       </c>
     </row>
@@ -776,76 +802,86 @@
           <t>BUG_REC_001</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Resume file upload allows double extension files (e.g., 'resume.pdf.doc') without explicit extension check</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Potential Defect / Exploratory Finding</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Resume file upload accepts double extension files (e.g., 'resume.pdf.doc') without explicit MIME-type verification</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Recruitment</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Demo</t>
-        </is>
-      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
+          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Public Demo</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
           <t>User is on Recruitment &gt; Add Candidate page.</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>1. Fill required candidate fields (Name, Email).
-2. Under Resume, select a file named 'sample_resume.pdf.doc'.
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>File Name: "sample_resume.pdf.doc" (Size: 250 KB)</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>1. Fill mandatory candidate fields (First Name, Last Name, Email).
+2. Under Resume upload, select file named 'sample_resume.pdf.doc'.
 3. Click 'Save' button.</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>System should strictly parse file extensions and verify MIME type before accepting multi-extension files.</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>System accepts the file attachment based solely on the final extension without MIME validation.</t>
-        </is>
-      </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>System should validate that file extensions are singular and verify file MIME type prior to acceptance.</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>System accepts the file because it only inspects the terminal extension (.doc), bypassing compound extension checks.</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J7" s="9" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>Always (100%)</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>TC_REC_008</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="P7" s="5" t="inlineStr">
         <is>
           <t>BUG_REC_001_double_extension.png</t>
         </is>
       </c>
-      <c r="O7" s="5" t="inlineStr">
-        <is>
-          <t>Minor security risk; file MIME-type verification recommended.</t>
+      <c r="Q7" s="5" t="inlineStr">
+        <is>
+          <t>Security and file handling exploratory observation.</t>
         </is>
       </c>
     </row>
@@ -855,77 +891,86 @@
           <t>BUG_LOGIN_001</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Simulated Defect (Lifecycle Demo)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Password input allows pasting plain text containing leading spaces without input sanitation warning</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Login</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Windows 11 / Edge v128 / OrangeHRM 5.x Demo</t>
-        </is>
-      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
+          <t>Windows 11 / Microsoft Edge v128 / OrangeHRM 5.x Public Demo</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
           <t>User is on the login page.</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>1. Copy ' admin123' (with a leading space) to clipboard.
-2. Paste into the Password field.
-3. Enter 'Admin' in Username.
-4. Click 'Login'.</t>
-        </is>
-      </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>System should either warn user about leading/trailing space in password or clarify authentication failure cause.</t>
+          <t>Username: "Admin", Password: " admin123" (with leading space)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>System displays generic 'Invalid credentials' banner without any indication of inadvertent whitespace.</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
+          <t>1. Copy ' admin123' (with leading space) to clipboard.
+2. Paste into Password field.
+3. Enter 'Admin' in Username and click 'Login'.</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Authentication should fail with standard message, but helper tooltip or trim behavior should guide user on whitespace.</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>System displays generic 'Invalid credentials' banner; retested in cycle 2 to verify strict character preservation.</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J8" s="9" t="inlineStr">
+      <c r="L8" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
         <is>
           <t>Always (100%)</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>Closed (Simulated)</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Closed (Simulated Fix &amp; Retest)</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>TC_LOGIN_002</t>
         </is>
       </c>
-      <c r="N8" s="5" t="inlineStr">
+      <c r="P8" s="5" t="inlineStr">
         <is>
           <t>BUG_LOGIN_001_password_space.png</t>
         </is>
       </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Retested in simulated cycle; verified standard behavior aligns with security best practices.</t>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>Simulated defect used to demonstrate full STLC Defect Lifecycle (New -&gt; Open -&gt; Fixed -&gt; Retest -&gt; Closed).</t>
         </is>
       </c>
     </row>
@@ -935,77 +980,86 @@
           <t>BUG_EMP_002</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Employee ID leading zeros stripped in table view causing visual discrepancy with search input</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Potential Defect / Exploratory Finding</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Employee ID leading zeros stripped in data table view causing visual discrepancy with search input</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Employee Management (PIM)</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Demo</t>
-        </is>
-      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Add employee with ID '0089'.</t>
+          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Public Demo</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>1. Navigate to PIM &gt; Add Employee.
-2. Enter names and specify Employee ID as '0089'.
-3. Click 'Save'.
-4. Search for '0089' in Employee List.</t>
+          <t>Add employee with custom ID '0089'.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Employee record in table should retain formatted leading zeros ('0089') as entered.</t>
+          <t>Employee ID: "0089", Names: "Test", "LeadingZero"</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>System strips leading zeros and renders ID as '89' in certain list views, requiring search for '89'.</t>
-        </is>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
+          <t>1. In PIM &gt; Add Employee, enter names and Employee ID '0089'.
+2. Click 'Save'.
+3. In Employee List, search for '0089'.</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Employee List table should display ID formatted as '0089', preserving user-entered leading zeros.</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>System strips leading zeros and renders ID as '89' in data table, requiring search query '89'.</t>
+        </is>
+      </c>
+      <c r="K9" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J9" s="9" t="inlineStr">
+      <c r="L9" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>Always (100%)</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>TC_EMP_007</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="P9" s="5" t="inlineStr">
         <is>
           <t>BUG_EMP_002_leading_zeros.png</t>
         </is>
       </c>
-      <c r="O9" s="5" t="inlineStr">
-        <is>
-          <t>Cosmetic/formatting defect in string handling.</t>
+      <c r="Q9" s="5" t="inlineStr">
+        <is>
+          <t>String versus integer datatype parsing discrepancy in UI table component.</t>
         </is>
       </c>
     </row>
@@ -1015,83 +1069,93 @@
           <t>BUG_REC_002</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Potential Defect / Exploratory Finding</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Candidate search by Vacancy does not reset results count text until full page reload</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Recruitment</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Demo</t>
-        </is>
-      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>User has performed a search in Recruitment &gt; Candidates.</t>
+          <t>Windows 11 / Chrome v128 / OrangeHRM 5.x Public Demo</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>1. Search candidates by a vacancy that yields 2 records.
+          <t>User has applied a search filter in Recruitment &gt; Candidates.</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Job Vacancy filter: Active Vacancy -&gt; Reset action</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>1. Search candidates by vacancy that yields 2 records.
 2. Click 'Reset' button.
-3. Observe '(2) Records Found' header label.</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>Records found counter should update dynamically to reflect total unfiltered candidate count upon clicking Reset.</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Table refreshes all records, but '(2) Records Found' label intermittently lags until manual browser reload.</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
+3. Observe '(2) Records Found' counter text.</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Counter text should dynamically update to reflect total unfiltered candidate count upon clicking Reset.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Data grid refreshes to display all candidates, but '(2) Records Found' text counter intermittently retains old count until page reload.</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="J10" s="9" t="inlineStr">
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>Intermittent (50%)</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>TC_REC_011</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="P10" s="5" t="inlineStr">
         <is>
           <t>BUG_REC_002_counter_lag.png</t>
         </is>
       </c>
-      <c r="O10" s="5" t="inlineStr">
-        <is>
-          <t>Minor UI synchronization issue in frontend state management.</t>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>Minor UI reactivity lag in Vue.js frontend state management.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Final audit and cleanup of OrangeHRM Manual Testing portfolio
</commit_message>
<xml_diff>
--- a/05-Defect-Management/Bug-Reports.xlsx
+++ b/05-Defect-Management/Bug-Reports.xlsx
@@ -804,7 +804,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Potential Defect / Exploratory Finding</t>
+          <t>Exploratory Finding</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Simulated Defect (Lifecycle Demo)</t>
+          <t>Simulated Defect</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -982,7 +982,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Potential Defect / Exploratory Finding</t>
+          <t>Exploratory Finding</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Potential Defect / Exploratory Finding</t>
+          <t>Exploratory Finding</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">

</xml_diff>